<commit_message>
SRIS-27: deleted descriptions of updateToPreviousForm, previousConfirmCode, mdardSoilVol from soil_relocation_source_site.xlsx / added descriptions of mlardYesNo into soil_relocation_source_site.xlsx
</commit_message>
<xml_diff>
--- a/fields_description/soil_relocation_source_sites.xlsx
+++ b/fields_description/soil_relocation_source_sites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28014"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB_REPOS\nr-soils-relocation\fields_description\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="13_ncr:1_{3ECF0116-F372-4A9E-9C3D-813C56CCA705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CD7F602-0CB0-49E1-B7AF-02D11C492F15}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF3E5DE8-087D-49DF-B54A-9EDAB3B3288A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,10 +41,19 @@
     <author>Roy Jeong</author>
   </authors>
   <commentList>
-    <comment ref="A41" authorId="0" shapeId="0" xr:uid="{BE0AFAC0-5342-4AD2-BD18-14851007C481}">
+    <comment ref="A39" authorId="0" shapeId="0" xr:uid="{BE0AFAC0-5342-4AD2-BD18-14851007C481}">
       <text>
-        <t>Roy Jeong:
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Roy Jeong:
 Never rename fields. The field name is not incorrect, it is currently actually referenced as such in AGOL internally.</t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -52,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
   <si>
     <t>field</t>
   </si>
@@ -66,18 +75,6 @@
     <t xml:space="preserve">The confirmation ID is a number generated by the CHEFS form each time a soil relocation notification form is submitted. The number is used by submitters, First Nations, municipalities, members of the public and ministry staff to track individual submissions. The confirmation ID can also be used to request additional information from the soil relocation team. </t>
   </si>
   <si>
-    <t>updateToPreviousForm</t>
-  </si>
-  <si>
-    <t>The field indicates whether the current soil relocation notification form is an update to a previous submission. Submitters must select 'Yes' if the form is an amendment or follow-up to an earlier submission, or 'No' if it is a new submission. This field is required and is recorded as 'Yes' or 'No' in the dataset to ensure clarity in tracking the status of soil relocation activities.</t>
-  </si>
-  <si>
-    <t>previousConfirmCode</t>
-  </si>
-  <si>
-    <t>The field is used when the current soil relocation notification form is an update to a previous submission. If the submitter selects 'Yes' to indicate that the form is an update, they must enter the confirmation code of the previous submission in this field. For example, a valid entry might be '105A2Z1A'. This code corresponds to the confirmation ID generated by the CHEFS form for the earlier submission, enabling accurate tracking and reference.</t>
-  </si>
-  <si>
     <t>ownerCompany</t>
   </si>
   <si>
@@ -252,12 +249,6 @@
     <t>The field records the soil volume to be relocated (in cubic metres) for the wildlands reverted (WLR) soil quality. The data is a numerical value, and an example entry might be '13579'.</t>
   </si>
   <si>
-    <t>mdardSoilVol</t>
-  </si>
-  <si>
-    <t>The field records the soil volume to be relocated (in cubic metres) for soil quality without potential for Metals Leaching/Acid Rock Drainage (ML/ARD) as evaluated under Protocol 19. The data is a numerical value, and an example entry might be '13579'.</t>
-  </si>
-  <si>
     <t>totalSoilVolume</t>
   </si>
   <si>
@@ -352,13 +343,19 @@
   </si>
   <si>
     <t>The field records the regional district of the second additional receiving site involved in the soil relocation. The data is a non-nullable text type. For example, 'Metro Vancouver Regional District.' is one of selections.</t>
+  </si>
+  <si>
+    <t>mlardYesNo</t>
+  </si>
+  <si>
+    <t>The field records whether the soil is composed of quarried material produced through the mining and crushing of bedrock. The data is stored as 'Yes' or 'No'.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -748,14 +745,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
     <col min="2" max="2" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -763,7 +760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -771,7 +768,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -779,7 +776,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -787,7 +784,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -795,15 +792,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -811,15 +808,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -827,7 +824,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -835,7 +832,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -843,7 +840,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -851,7 +848,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -859,7 +856,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -867,7 +864,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -875,7 +872,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -883,7 +880,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -891,7 +888,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -899,7 +896,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -907,7 +904,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
@@ -915,31 +912,31 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>42</v>
       </c>
       <c r="B22" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -947,7 +944,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -955,7 +952,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -963,7 +960,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -971,7 +968,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -979,7 +976,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>56</v>
       </c>
@@ -987,7 +984,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -995,7 +992,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -1003,7 +1000,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -1011,148 +1008,132 @@
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>64</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
-      <c r="A34" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>66</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
-      <c r="A35" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>68</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
-      <c r="A36" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>70</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
-      <c r="A37" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>72</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
-      <c r="A38" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>74</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
-      <c r="A39" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>76</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
-      <c r="A40" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>78</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
-      <c r="A41" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>80</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
-      <c r="A42" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>82</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
-      <c r="A43" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>84</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
-      <c r="A44" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>86</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
-      <c r="A45" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>88</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
-      <c r="A46" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>90</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
-      <c r="A47" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>92</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2">
-      <c r="A48" t="s">
-        <v>94</v>
-      </c>
-      <c r="B48" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B49" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
-        <v>98</v>
-      </c>
-      <c r="B50" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>